<commit_message>
feat: add unsubmitted-first sorting on admin applications
</commit_message>
<xml_diff>
--- a/samples/user-import-sample２.xlsx
+++ b/samples/user-import-sample２.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OPAthird01\Projects\after-school-day-service\samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8DD87E9-95D8-41D0-BF23-CCF716D91C1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9FC704D-C1BB-4C2E-88AE-268A4D71ADEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="利用者" sheetId="1" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="968" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="278">
   <si>
     <t>login_id</t>
   </si>
@@ -1832,21 +1832,6 @@
     <phoneticPr fontId="0"/>
   </si>
   <si>
-    <t>サード・チャレンジ</t>
-  </si>
-  <si>
-    <t>サード・アスリート</t>
-  </si>
-  <si>
-    <t>ネクスト・サード</t>
-  </si>
-  <si>
-    <t>サード・ネクスト</t>
-  </si>
-  <si>
-    <t>セカンド・チャレンジ</t>
-  </si>
-  <si>
     <t>オーパ|オーパ|チャレンジ|ステップ|オーパ|ステップ</t>
   </si>
   <si>
@@ -1961,12 +1946,6 @@
     <t>サード|サード|サード|アスリート|サード|アスリート</t>
   </si>
   <si>
-    <t>チャレンジ|サード・チャレンジ</t>
-  </si>
-  <si>
-    <t>サード|サード・チャレンジ</t>
-  </si>
-  <si>
     <t>サード|サード|サード|ネクスト|チャレンジ</t>
   </si>
   <si>
@@ -1977,9 +1956,6 @@
   </si>
   <si>
     <t>サード|サード|サード|サード</t>
-  </si>
-  <si>
-    <t>サード|アスリート|サード・アスリート</t>
   </si>
   <si>
     <t>サード|サード|サード|サード|サード</t>
@@ -2119,6 +2095,24 @@
   <si>
     <t>management_no</t>
     <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>サード</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>セカンド</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>アスリート</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>チャレンジ|サード</t>
+  </si>
+  <si>
+    <t>サード|アスリート|サード</t>
   </si>
 </sst>
 </file>
@@ -2586,6 +2580,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N230"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="8" max="13" width="20.375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
@@ -2601,7 +2598,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -2684,7 +2681,7 @@
         <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="E3">
         <v>9002</v>
@@ -2729,7 +2726,7 @@
         <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="E4">
         <v>9003</v>
@@ -2771,7 +2768,7 @@
         <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="E5">
         <v>9004</v>
@@ -2804,7 +2801,7 @@
         <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="E6">
         <v>9005</v>
@@ -2837,7 +2834,7 @@
         <v>23</v>
       </c>
       <c r="D7" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="E7">
         <v>9006</v>
@@ -2879,7 +2876,7 @@
         <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="E8">
         <v>9007</v>
@@ -2918,7 +2915,7 @@
         <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="E9">
         <v>9008</v>
@@ -2957,7 +2954,7 @@
         <v>23</v>
       </c>
       <c r="D10" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="E10">
         <v>9009</v>
@@ -2996,7 +2993,7 @@
         <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="E11">
         <v>9010</v>
@@ -3035,7 +3032,7 @@
         <v>15</v>
       </c>
       <c r="D12" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="E12">
         <v>9011</v>
@@ -3071,7 +3068,7 @@
         <v>23</v>
       </c>
       <c r="D13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="E13">
         <v>9012</v>
@@ -3113,7 +3110,7 @@
         <v>18</v>
       </c>
       <c r="D14" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="E14">
         <v>9013</v>
@@ -3149,7 +3146,7 @@
         <v>23</v>
       </c>
       <c r="D15" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="E15">
         <v>9014</v>
@@ -3188,7 +3185,7 @@
         <v>14</v>
       </c>
       <c r="D16" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="E16">
         <v>9015</v>
@@ -3218,7 +3215,7 @@
         <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="E17">
         <v>9016</v>
@@ -3248,7 +3245,7 @@
         <v>23</v>
       </c>
       <c r="D18" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="E18">
         <v>9017</v>
@@ -3278,7 +3275,7 @@
         <v>11</v>
       </c>
       <c r="D19" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="E19">
         <v>9018</v>
@@ -3308,7 +3305,7 @@
         <v>16</v>
       </c>
       <c r="D20" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="E20">
         <v>9019</v>
@@ -3341,7 +3338,7 @@
         <v>23</v>
       </c>
       <c r="D21" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="E21">
         <v>9020</v>
@@ -3374,7 +3371,7 @@
         <v>23</v>
       </c>
       <c r="D22" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="E22">
         <v>9021</v>
@@ -3416,7 +3413,7 @@
         <v>19</v>
       </c>
       <c r="D23" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="E23">
         <v>9022</v>
@@ -3455,7 +3452,7 @@
         <v>23</v>
       </c>
       <c r="D24" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="E24">
         <v>9023</v>
@@ -3494,7 +3491,7 @@
         <v>23</v>
       </c>
       <c r="D25" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="E25">
         <v>9024</v>
@@ -3536,7 +3533,7 @@
         <v>13</v>
       </c>
       <c r="D26" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="E26">
         <v>9025</v>
@@ -3569,7 +3566,7 @@
         <v>20</v>
       </c>
       <c r="D27" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="E27">
         <v>9026</v>
@@ -3611,7 +3608,7 @@
         <v>23</v>
       </c>
       <c r="D28" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E28">
         <v>9027</v>
@@ -3653,7 +3650,7 @@
         <v>23</v>
       </c>
       <c r="D29" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="E29">
         <v>9028</v>
@@ -3692,7 +3689,7 @@
         <v>20</v>
       </c>
       <c r="D30" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="E30">
         <v>9029</v>
@@ -3731,7 +3728,7 @@
         <v>23</v>
       </c>
       <c r="D31" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="E31">
         <v>9030</v>
@@ -3773,7 +3770,7 @@
         <v>14</v>
       </c>
       <c r="D32" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="E32">
         <v>9031</v>
@@ -3806,7 +3803,7 @@
         <v>23</v>
       </c>
       <c r="D33" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="E33">
         <v>9032</v>
@@ -3845,7 +3842,7 @@
         <v>15</v>
       </c>
       <c r="D34" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="E34">
         <v>9033</v>
@@ -3878,7 +3875,7 @@
         <v>10</v>
       </c>
       <c r="D35" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="E35">
         <v>9034</v>
@@ -3908,7 +3905,7 @@
         <v>10</v>
       </c>
       <c r="D36" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="E36">
         <v>9035</v>
@@ -3938,7 +3935,7 @@
         <v>20</v>
       </c>
       <c r="D37" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="E37">
         <v>9036</v>
@@ -3977,7 +3974,7 @@
         <v>23</v>
       </c>
       <c r="D38" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E38">
         <v>9037</v>
@@ -4019,7 +4016,7 @@
         <v>23</v>
       </c>
       <c r="D39" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="E39">
         <v>9038</v>
@@ -4058,7 +4055,7 @@
         <v>13</v>
       </c>
       <c r="D40" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="E40">
         <v>9039</v>
@@ -4091,7 +4088,7 @@
         <v>20</v>
       </c>
       <c r="D41" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="E41">
         <v>9040</v>
@@ -4130,7 +4127,7 @@
         <v>23</v>
       </c>
       <c r="D42" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="E42">
         <v>9041</v>
@@ -4199,7 +4196,7 @@
         <v>20</v>
       </c>
       <c r="D44" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="E44">
         <v>9043</v>
@@ -4238,7 +4235,7 @@
         <v>23</v>
       </c>
       <c r="D45" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="E45">
         <v>9044</v>
@@ -4277,7 +4274,7 @@
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="E46">
         <v>9045</v>
@@ -4316,7 +4313,7 @@
         <v>20</v>
       </c>
       <c r="D47" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E47">
         <v>9046</v>
@@ -4358,7 +4355,7 @@
         <v>20</v>
       </c>
       <c r="D48" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="E48">
         <v>9047</v>
@@ -4388,7 +4385,7 @@
         <v>23</v>
       </c>
       <c r="D49" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="E49">
         <v>9048</v>
@@ -4430,7 +4427,7 @@
         <v>20</v>
       </c>
       <c r="D50" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="E50">
         <v>9049</v>
@@ -4493,7 +4490,7 @@
         <v>23</v>
       </c>
       <c r="D52" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="E52">
         <v>9051</v>
@@ -4535,7 +4532,7 @@
         <v>23</v>
       </c>
       <c r="D53" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="E53">
         <v>9052</v>
@@ -4577,7 +4574,7 @@
         <v>23</v>
       </c>
       <c r="D54" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="E54">
         <v>9053</v>
@@ -4619,7 +4616,7 @@
         <v>20</v>
       </c>
       <c r="D55" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="E55">
         <v>9054</v>
@@ -4658,7 +4655,7 @@
         <v>23</v>
       </c>
       <c r="D56" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="E56">
         <v>9055</v>
@@ -4700,7 +4697,7 @@
         <v>23</v>
       </c>
       <c r="D57" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="E57">
         <v>9056</v>
@@ -4742,7 +4739,7 @@
         <v>10</v>
       </c>
       <c r="D58" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="E58">
         <v>9057</v>
@@ -4772,7 +4769,7 @@
         <v>8</v>
       </c>
       <c r="D59" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="E59">
         <v>9058</v>
@@ -4802,7 +4799,7 @@
         <v>14</v>
       </c>
       <c r="D60" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="E60">
         <v>9059</v>
@@ -4832,7 +4829,7 @@
         <v>23</v>
       </c>
       <c r="D61" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="E61">
         <v>9060</v>
@@ -4874,7 +4871,7 @@
         <v>23</v>
       </c>
       <c r="D62" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="E62">
         <v>9061</v>
@@ -4916,7 +4913,7 @@
         <v>10</v>
       </c>
       <c r="D63" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="E63">
         <v>9062</v>
@@ -4958,7 +4955,7 @@
         <v>15</v>
       </c>
       <c r="D64" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="E64">
         <v>9063</v>
@@ -4994,7 +4991,7 @@
         <v>15</v>
       </c>
       <c r="D65" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="E65">
         <v>9064</v>
@@ -5027,7 +5024,7 @@
         <v>23</v>
       </c>
       <c r="D66" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="E66">
         <v>9065</v>
@@ -5060,7 +5057,7 @@
         <v>23</v>
       </c>
       <c r="D67" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="E67">
         <v>9066</v>
@@ -5096,7 +5093,7 @@
         <v>10</v>
       </c>
       <c r="D68" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="E68">
         <v>9067</v>
@@ -5138,7 +5135,7 @@
         <v>23</v>
       </c>
       <c r="D69" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="E69">
         <v>9068</v>
@@ -5180,7 +5177,7 @@
         <v>10</v>
       </c>
       <c r="D70" t="s">
-        <v>228</v>
+        <v>276</v>
       </c>
       <c r="E70">
         <v>9069</v>
@@ -5192,11 +5189,11 @@
         <v>21</v>
       </c>
       <c r="M70" t="s">
-        <v>185</v>
+        <v>273</v>
       </c>
       <c r="N70" t="str" cm="1">
         <f t="array" ref="N70">_xlfn.TEXTJOIN("|",TRUE,_xlfn.UNIQUE(_xlfn._xlws.FILTER(H70:M70,H70:M70&lt;&gt;"")))</f>
-        <v>チャレンジ|サード・チャレンジ</v>
+        <v>チャレンジ|サード</v>
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.15">
@@ -5210,7 +5207,7 @@
         <v>10</v>
       </c>
       <c r="D71" t="s">
-        <v>185</v>
+        <v>17</v>
       </c>
       <c r="E71">
         <v>9070</v>
@@ -5218,12 +5215,12 @@
       <c r="F71">
         <v>7196</v>
       </c>
-      <c r="J71" t="s">
-        <v>185</v>
+      <c r="M71" t="s">
+        <v>273</v>
       </c>
       <c r="N71" t="str" cm="1">
         <f t="array" ref="N71">_xlfn.TEXTJOIN("|",TRUE,_xlfn.UNIQUE(_xlfn._xlws.FILTER(H71:M71,H71:M71&lt;&gt;"")))</f>
-        <v>サード・チャレンジ</v>
+        <v>サード</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.15">
@@ -5237,7 +5234,7 @@
         <v>9</v>
       </c>
       <c r="D72" t="s">
-        <v>229</v>
+        <v>216</v>
       </c>
       <c r="E72">
         <v>9071</v>
@@ -5249,11 +5246,11 @@
         <v>17</v>
       </c>
       <c r="M72" t="s">
-        <v>185</v>
+        <v>273</v>
       </c>
       <c r="N72" t="str" cm="1">
         <f t="array" ref="N72">_xlfn.TEXTJOIN("|",TRUE,_xlfn.UNIQUE(_xlfn._xlws.FILTER(H72:M72,H72:M72&lt;&gt;"")))</f>
-        <v>サード|サード・チャレンジ</v>
+        <v>サード|サード</v>
       </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.15">
@@ -5267,7 +5264,7 @@
         <v>23</v>
       </c>
       <c r="D73" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="E73">
         <v>9072</v>
@@ -5306,7 +5303,7 @@
         <v>20</v>
       </c>
       <c r="D74" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="E74">
         <v>9073</v>
@@ -5345,7 +5342,7 @@
         <v>23</v>
       </c>
       <c r="D75" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="E75">
         <v>9074</v>
@@ -5387,7 +5384,7 @@
         <v>10</v>
       </c>
       <c r="D76" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="E76">
         <v>9075</v>
@@ -5417,7 +5414,7 @@
         <v>10</v>
       </c>
       <c r="D77" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="E77">
         <v>9076</v>
@@ -5447,7 +5444,7 @@
         <v>20</v>
       </c>
       <c r="D78" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="E78">
         <v>9077</v>
@@ -5483,7 +5480,7 @@
         <v>23</v>
       </c>
       <c r="D79" t="s">
-        <v>234</v>
+        <v>277</v>
       </c>
       <c r="E79">
         <v>9078</v>
@@ -5498,11 +5495,11 @@
         <v>19</v>
       </c>
       <c r="M79" t="s">
-        <v>186</v>
+        <v>273</v>
       </c>
       <c r="N79" t="str" cm="1">
         <f t="array" ref="N79">_xlfn.TEXTJOIN("|",TRUE,_xlfn.UNIQUE(_xlfn._xlws.FILTER(H79:M79,H79:M79&lt;&gt;"")))</f>
-        <v>サード|アスリート|サード・アスリート</v>
+        <v>サード|アスリート|サード</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.15">
@@ -5516,7 +5513,7 @@
         <v>23</v>
       </c>
       <c r="D80" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="E80">
         <v>9079</v>
@@ -5555,7 +5552,7 @@
         <v>20</v>
       </c>
       <c r="D81" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="E81">
         <v>9080</v>
@@ -5594,7 +5591,7 @@
         <v>27</v>
       </c>
       <c r="D82" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="E82">
         <v>9081</v>
@@ -5636,7 +5633,7 @@
         <v>10</v>
       </c>
       <c r="D83" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="E83">
         <v>9082</v>
@@ -5666,7 +5663,7 @@
         <v>10</v>
       </c>
       <c r="D84" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="E84">
         <v>9083</v>
@@ -5696,7 +5693,7 @@
         <v>27</v>
       </c>
       <c r="D85" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="E85">
         <v>9084</v>
@@ -5765,7 +5762,7 @@
         <v>27</v>
       </c>
       <c r="D87" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="E87">
         <v>9086</v>
@@ -5807,7 +5804,7 @@
         <v>23</v>
       </c>
       <c r="D88" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="E88">
         <v>9087</v>
@@ -5849,7 +5846,7 @@
         <v>18</v>
       </c>
       <c r="D89" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="E89">
         <v>9088</v>
@@ -5891,7 +5888,7 @@
         <v>19</v>
       </c>
       <c r="D90" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="E90">
         <v>9089</v>
@@ -5933,7 +5930,7 @@
         <v>23</v>
       </c>
       <c r="D91" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="E91">
         <v>9090</v>
@@ -5972,7 +5969,7 @@
         <v>27</v>
       </c>
       <c r="D92" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="E92">
         <v>9091</v>
@@ -6014,7 +6011,7 @@
         <v>23</v>
       </c>
       <c r="D93" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="E93">
         <v>9092</v>
@@ -6056,7 +6053,7 @@
         <v>5</v>
       </c>
       <c r="D94" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="E94">
         <v>9093</v>
@@ -6089,7 +6086,7 @@
         <v>10</v>
       </c>
       <c r="D95" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="E95">
         <v>9094</v>
@@ -6119,7 +6116,7 @@
         <v>11</v>
       </c>
       <c r="D96" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="E96">
         <v>9095</v>
@@ -6149,7 +6146,7 @@
         <v>23</v>
       </c>
       <c r="D97" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="E97">
         <v>9096</v>
@@ -6182,7 +6179,7 @@
         <v>8</v>
       </c>
       <c r="D98" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="E98">
         <v>9097</v>
@@ -6212,7 +6209,7 @@
         <v>15</v>
       </c>
       <c r="D99" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="E99">
         <v>9098</v>
@@ -6296,7 +6293,7 @@
         <v>22</v>
       </c>
       <c r="D102" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="E102">
         <v>9101</v>
@@ -6335,7 +6332,7 @@
         <v>14</v>
       </c>
       <c r="D103" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="E103">
         <v>9102</v>
@@ -6368,7 +6365,7 @@
         <v>23</v>
       </c>
       <c r="D104" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="E104">
         <v>9103</v>
@@ -6410,7 +6407,7 @@
         <v>23</v>
       </c>
       <c r="D105" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="E105">
         <v>9104</v>
@@ -6449,7 +6446,7 @@
         <v>10</v>
       </c>
       <c r="D106" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="E106">
         <v>9105</v>
@@ -6479,7 +6476,7 @@
         <v>20</v>
       </c>
       <c r="D107" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="E107">
         <v>9106</v>
@@ -6521,7 +6518,7 @@
         <v>23</v>
       </c>
       <c r="D108" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="E108">
         <v>9107</v>
@@ -6560,7 +6557,7 @@
         <v>20</v>
       </c>
       <c r="D109" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="E109">
         <v>9108</v>
@@ -6593,7 +6590,7 @@
         <v>9</v>
       </c>
       <c r="D110" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="E110">
         <v>9109</v>
@@ -6626,7 +6623,7 @@
         <v>23</v>
       </c>
       <c r="D111" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="E111">
         <v>9110</v>
@@ -6662,7 +6659,7 @@
         <v>10</v>
       </c>
       <c r="D112" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="E112">
         <v>9111</v>
@@ -6692,7 +6689,7 @@
         <v>10</v>
       </c>
       <c r="D113" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="E113">
         <v>9112</v>
@@ -6749,7 +6746,7 @@
         <v>23</v>
       </c>
       <c r="D115" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="E115">
         <v>9114</v>
@@ -6815,7 +6812,7 @@
         <v>23</v>
       </c>
       <c r="D117" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="E117">
         <v>9116</v>
@@ -6851,7 +6848,7 @@
         <v>4</v>
       </c>
       <c r="D118" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="E118">
         <v>9117</v>
@@ -6893,7 +6890,7 @@
         <v>13</v>
       </c>
       <c r="D119" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="E119">
         <v>9118</v>
@@ -6926,7 +6923,7 @@
         <v>21</v>
       </c>
       <c r="D120" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="E120">
         <v>9119</v>
@@ -6965,7 +6962,7 @@
         <v>23</v>
       </c>
       <c r="D121" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="E121">
         <v>9120</v>
@@ -6998,7 +6995,7 @@
         <v>18</v>
       </c>
       <c r="D122" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="E122">
         <v>9121</v>
@@ -7034,7 +7031,7 @@
         <v>14</v>
       </c>
       <c r="D123" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="E123">
         <v>9122</v>
@@ -7067,7 +7064,7 @@
         <v>23</v>
       </c>
       <c r="D124" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="E124">
         <v>9123</v>
@@ -7106,7 +7103,7 @@
         <v>15</v>
       </c>
       <c r="D125" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="E125">
         <v>9124</v>
@@ -7142,7 +7139,7 @@
         <v>23</v>
       </c>
       <c r="D126" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="E126">
         <v>9125</v>
@@ -7181,7 +7178,7 @@
         <v>20</v>
       </c>
       <c r="D127" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="E127">
         <v>9126</v>
@@ -7223,7 +7220,7 @@
         <v>15</v>
       </c>
       <c r="D128" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="E128">
         <v>9127</v>
@@ -7244,11 +7241,11 @@
         <v>18</v>
       </c>
       <c r="M128" t="s">
-        <v>187</v>
+        <v>273</v>
       </c>
       <c r="N128" t="str" cm="1">
         <f t="array" ref="N128">_xlfn.TEXTJOIN("|",TRUE,_xlfn.UNIQUE(_xlfn._xlws.FILTER(H128:M128,H128:M128&lt;&gt;"")))</f>
-        <v>ネクスト|サード|サード|ネクスト|ネクスト・サード</v>
+        <v>ネクスト|サード|サード|ネクスト|サード</v>
       </c>
     </row>
     <row r="129" spans="1:14" x14ac:dyDescent="0.15">
@@ -7262,7 +7259,7 @@
         <v>15</v>
       </c>
       <c r="D129" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="E129">
         <v>9128</v>
@@ -7280,11 +7277,11 @@
         <v>18</v>
       </c>
       <c r="M129" t="s">
-        <v>188</v>
+        <v>273</v>
       </c>
       <c r="N129" t="str" cm="1">
         <f t="array" ref="N129">_xlfn.TEXTJOIN("|",TRUE,_xlfn.UNIQUE(_xlfn._xlws.FILTER(H129:M129,H129:M129&lt;&gt;"")))</f>
-        <v>ネクスト|サード|ネクスト|サード・ネクスト</v>
+        <v>ネクスト|サード|ネクスト|サード</v>
       </c>
     </row>
     <row r="130" spans="1:14" x14ac:dyDescent="0.15">
@@ -7298,7 +7295,7 @@
         <v>20</v>
       </c>
       <c r="D130" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="E130">
         <v>9129</v>
@@ -7340,7 +7337,7 @@
         <v>23</v>
       </c>
       <c r="D131" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="E131">
         <v>9130</v>
@@ -7400,7 +7397,7 @@
         <v>23</v>
       </c>
       <c r="D133" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="E133">
         <v>9132</v>
@@ -7439,7 +7436,7 @@
         <v>15</v>
       </c>
       <c r="D134" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="E134">
         <v>9133</v>
@@ -7475,7 +7472,7 @@
         <v>23</v>
       </c>
       <c r="D135" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="E135">
         <v>9134</v>
@@ -7517,7 +7514,7 @@
         <v>21</v>
       </c>
       <c r="D136" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="E136">
         <v>9135</v>
@@ -7559,7 +7556,7 @@
         <v>15</v>
       </c>
       <c r="D137" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="E137">
         <v>9136</v>
@@ -7592,7 +7589,7 @@
         <v>21</v>
       </c>
       <c r="D138" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="E138">
         <v>9137</v>
@@ -7634,7 +7631,7 @@
         <v>23</v>
       </c>
       <c r="D139" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="E139">
         <v>9138</v>
@@ -7670,7 +7667,7 @@
         <v>20</v>
       </c>
       <c r="D140" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="E140">
         <v>9139</v>
@@ -7685,11 +7682,11 @@
         <v>21</v>
       </c>
       <c r="M140" t="s">
-        <v>189</v>
+        <v>274</v>
       </c>
       <c r="N140" t="str" cm="1">
         <f t="array" ref="N140">_xlfn.TEXTJOIN("|",TRUE,_xlfn.UNIQUE(_xlfn._xlws.FILTER(H140:M140,H140:M140&lt;&gt;"")))</f>
-        <v>セカンド|チャレンジ|セカンド・チャレンジ</v>
+        <v>セカンド|チャレンジ|セカンド</v>
       </c>
     </row>
     <row r="141" spans="1:14" x14ac:dyDescent="0.15">
@@ -7730,7 +7727,7 @@
         <v>15</v>
       </c>
       <c r="D142" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="E142">
         <v>9141</v>
@@ -7790,7 +7787,7 @@
         <v>10</v>
       </c>
       <c r="D144" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="E144">
         <v>9143</v>
@@ -7823,7 +7820,7 @@
         <v>23</v>
       </c>
       <c r="D145" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="E145">
         <v>9144</v>
@@ -7940,7 +7937,7 @@
         <v>21</v>
       </c>
       <c r="D149" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="E149">
         <v>9148</v>
@@ -7976,7 +7973,7 @@
         <v>23</v>
       </c>
       <c r="D150" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="E150">
         <v>9149</v>
@@ -8012,7 +8009,7 @@
         <v>15</v>
       </c>
       <c r="D151" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="E151">
         <v>9150</v>
@@ -8069,7 +8066,7 @@
         <v>23</v>
       </c>
       <c r="D153" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="E153">
         <v>9152</v>
@@ -8111,7 +8108,7 @@
         <v>15</v>
       </c>
       <c r="D154" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="E154">
         <v>9153</v>
@@ -8141,7 +8138,7 @@
         <v>19</v>
       </c>
       <c r="D155" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="E155">
         <v>9154</v>
@@ -8182,8 +8179,8 @@
       <c r="C156">
         <v>23</v>
       </c>
-      <c r="D156" t="e" vm="1">
-        <v>#VALUE!</v>
+      <c r="D156" t="s">
+        <v>275</v>
       </c>
       <c r="E156">
         <v>9155</v>
@@ -8207,7 +8204,7 @@
         <v>11</v>
       </c>
       <c r="D157" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="E157">
         <v>9156</v>
@@ -8264,7 +8261,7 @@
         <v>15</v>
       </c>
       <c r="D159" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="E159">
         <v>9158</v>
@@ -8297,7 +8294,7 @@
         <v>20</v>
       </c>
       <c r="D160" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="E160">
         <v>9159</v>
@@ -8332,6 +8329,9 @@
       <c r="C161">
         <v>10</v>
       </c>
+      <c r="D161" t="s">
+        <v>270</v>
+      </c>
       <c r="E161">
         <v>9160</v>
       </c>
@@ -8353,6 +8353,9 @@
       <c r="C162">
         <v>0</v>
       </c>
+      <c r="D162" t="s">
+        <v>270</v>
+      </c>
       <c r="E162">
         <v>9161</v>
       </c>
@@ -8374,6 +8377,9 @@
       <c r="C163">
         <v>5</v>
       </c>
+      <c r="D163" t="s">
+        <v>270</v>
+      </c>
       <c r="E163">
         <v>9162</v>
       </c>
@@ -8395,6 +8401,9 @@
       <c r="C164">
         <v>0</v>
       </c>
+      <c r="D164" t="s">
+        <v>270</v>
+      </c>
       <c r="E164">
         <v>9163</v>
       </c>
@@ -8414,7 +8423,7 @@
         <v>184</v>
       </c>
       <c r="D165" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="E165">
         <v>9164</v>

</xml_diff>